<commit_message>
updates including mostly style
</commit_message>
<xml_diff>
--- a/cv/cv_data.xlsx
+++ b/cv/cv_data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10719"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10222"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sjspielman/sjspielman.github.io/cv/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA2C4A47-B18E-874A-8A57-4DF46C6307B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F246A502-6CB1-CB47-9EE7-66C7DED3F3EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-36500" yWindow="-100" windowWidth="35560" windowHeight="16300" activeTab="2" xr2:uid="{F213A91E-98B5-B244-B12A-A608C8962BCD}"/>
+    <workbookView xWindow="4580" yWindow="4640" windowWidth="35560" windowHeight="16300" activeTab="1" xr2:uid="{F213A91E-98B5-B244-B12A-A608C8962BCD}"/>
   </bookViews>
   <sheets>
     <sheet name="education" sheetId="10" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="47">
   <si>
     <t>institution</t>
   </si>
@@ -163,16 +163,19 @@
     <t>Inf</t>
   </si>
   <si>
-    <t>Develop open-source tools and data repositories, and lead training workshops to support pediatric cancer researchers</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Developed research in methods for quantifying protein evolution and taught graduate-level courses in Biostatistics and Evolutionary Medicine. </t>
-  </si>
-  <si>
     <t xml:space="preserve">Computational molecular evolution research, including phylogenetic modeling and virus evolution. </t>
   </si>
   <si>
     <t>Data Scientist, Childhood Cancer Data Lab</t>
+  </si>
+  <si>
+    <t>Developed research in methods for quantifying protein evolution and taught graduate-level courses in Biostatistics and Evolutionary Medicine</t>
+  </si>
+  <si>
+    <t>Ran undergraduate research lab focused on methods in molecular evolution and developed undegradute-level courses in Evolutionary Biology and Data Science</t>
+  </si>
+  <si>
+    <t>Develop open-source tools, data repositories, and training workshops to accelerate pediatric cancer research</t>
   </si>
 </sst>
 </file>
@@ -260,9 +263,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -300,7 +303,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -406,7 +409,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -548,7 +551,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -679,7 +682,7 @@
         <v>17</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.2">
@@ -725,7 +728,7 @@
         <v>23</v>
       </c>
       <c r="G4" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.2">
@@ -747,10 +750,13 @@
       <c r="F5" t="s">
         <v>27</v>
       </c>
+      <c r="G5" t="s">
+        <v>45</v>
+      </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>28</v>
@@ -768,7 +774,7 @@
         <v>30</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">

</xml_diff>